<commit_message>
updated testplan with cg info
</commit_message>
<xml_diff>
--- a/LED_MUX_CONTROLLER_testplan.xlsx
+++ b/LED_MUX_CONTROLLER_testplan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestPlan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="TestPlan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -690,7 +690,7 @@
 3) Read 0x4004 expect Done=0.
 4) Read 0x4008 expect 0.
 Constraints: No APB traffic during reset assert.
-Checkers: SCB-1, SCB-2, SCB-3; assert_sel_out_reset_value, assert_seg_out_reset_value.</t>
+Checkers: SCB-1, SCB-2, SCB-3; assert_sel_out_reset_value, assert_seg_out_reset_value; COV cg_enable.default_at_reset, cg_done.bin_0.</t>
         </is>
       </c>
       <c r="F4" s="18" t="inlineStr">
@@ -698,7 +698,11 @@
           <t>assert_sel_out_reset_value, assert_seg_out_reset_value</t>
         </is>
       </c>
-      <c r="G4" s="18" t="inlineStr"/>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>cg_enable, cg_done</t>
+        </is>
+      </c>
       <c r="H4" s="18" t="inlineStr">
         <is>
           <t>line, branch</t>
@@ -735,7 +739,7 @@
 3) Write 0x4000=1.
 4) Read 0x4000.
 Constraints: wdata[0] only (FR 3.4, §4.3).
-Checkers: SCB-1; COV cg_enable.</t>
+Checkers: SCB-1; COV cg_enable (cp_led_enable, cp_enable_trans).</t>
         </is>
       </c>
       <c r="F5" s="18" t="inlineStr"/>
@@ -1293,7 +1297,7 @@
 3) Poll Done.
 4) Scoreboard compare digits 0,0,0,0,4,2.
 Constraints: error_q==42; C-4 hold, C-5 latency (AC-B1).
-Checkers: SCB-4, SCB-5, SCB-6, SCB-8; assert_sel_out_onehot_active_low, assert_seg_out_bit7_always_one, check_60_80_cycle; COV cg_digits, cg_error_q.</t>
+Checkers: SCB-4, SCB-5, SCB-6, SCB-8; assert_sel_out_onehot_active_low, assert_seg_out_bit7_always_one, check_60_80_cycle; COV cg_error_q, cg_digits (cp_digit_pos, cp_digit_val).</t>
         </is>
       </c>
       <c r="F18" s="18" t="inlineStr">
@@ -1303,7 +1307,7 @@
       </c>
       <c r="G18" s="18" t="inlineStr">
         <is>
-          <t>cg_digits, cg_error_q</t>
+          <t>cg_error_q, cg_digits</t>
         </is>
       </c>
       <c r="H18" s="18" t="inlineStr">
@@ -1573,7 +1577,7 @@
 2) Poll Done.
 3) Expect display 000001.
 Constraints: Golden = error_q % 1_000_000 (FR 3.6, C-3, AC-B4).
-Checkers: SCB-9; assert_sel_out_onehot_active_low, assert_seg_out_bit7_always_one; COV cg_overflow, cg_digits.</t>
+Checkers: SCB-9; assert_sel_out_onehot_active_low, assert_seg_out_bit7_always_one; COV cg_overflow, cg_error_q overflow bins.</t>
         </is>
       </c>
       <c r="F24" s="18" t="inlineStr">
@@ -1583,7 +1587,7 @@
       </c>
       <c r="G24" s="18" t="inlineStr">
         <is>
-          <t>cg_overflow, cg_digits</t>
+          <t>cg_overflow, cg_error_q</t>
         </is>
       </c>
       <c r="H24" s="18" t="inlineStr">
@@ -1707,7 +1711,7 @@
 2) Drive error_q=55.
 3) Confirm seg_out does not update.
 Constraints: LED_enable==0 (FR 3.4, AC-E2).
-Checkers: SCB-7; COV cg_enable.</t>
+Checkers: SCB-7; COV cg_enable (bin_off, on_to_off).</t>
         </is>
       </c>
       <c r="F27" s="18" t="inlineStr"/>
@@ -1955,7 +1959,7 @@
         <is>
           <t>1) For d in 0..9: drive error_q with ones digit d; poll Done; compare encoding.
 Constraints: 10 iterations (AC-C1, AC-B1).
-Checkers: SCB-5; cover_seg_out_decimal_digit; COV cg_digits.</t>
+Checkers: SCB-5; cover_seg_out_decimal_digit; COV cg_digits, cx_digit_pos_x_digit_val.</t>
         </is>
       </c>
       <c r="F33" s="18" t="inlineStr">
@@ -1965,7 +1969,7 @@
       </c>
       <c r="G33" s="18" t="inlineStr">
         <is>
-          <t>cg_digits</t>
+          <t>cg_digits, cx_digit_pos_x_digit_val</t>
         </is>
       </c>
       <c r="H33" s="18" t="inlineStr">
@@ -2009,7 +2013,7 @@
 4) Poll Done.
 5) Scoreboard pass.
 Constraints: error_q=42.
-Checkers: SCB-1..9; assert_sel_out_reset_value, assert_seg_out_reset_value, assert_sel_out_onehot_active_low, assert_seg_out_bit7_always_one, assert_apb_setup_phase, assert_apb_access_phase, assert_apb_pready_complete, assert_apb_pslerr_invalid_addr, cover_sel_out_digit_position, cover_seg_out_decimal_digit, check_60_80_cycle, check_hold_1002_cycle; COV all.</t>
+Checkers: SCB-1..9; assert_sel_out_reset_value, assert_seg_out_reset_value, assert_sel_out_onehot_active_low, assert_seg_out_bit7_always_one, assert_apb_setup_phase, assert_apb_access_phase, assert_apb_pready_complete, assert_apb_pslerr_invalid_addr, cover_sel_out_digit_position, cover_seg_out_decimal_digit, check_60_80_cycle, check_hold_1002_cycle; COV cg_enable, cg_done, cg_error_q, cg_digits, cg_overflow.</t>
         </is>
       </c>
       <c r="F34" s="18" t="inlineStr">
@@ -2019,7 +2023,7 @@
       </c>
       <c r="G34" s="18" t="inlineStr">
         <is>
-          <t>cg_error_q, cg_digits, cg_enable, cg_done, cg_overflow</t>
+          <t>cg_enable, cg_done, cg_error_q, cg_digits, cg_overflow</t>
         </is>
       </c>
       <c r="H34" s="18" t="inlineStr">

</xml_diff>